<commit_message>
Update reports 2026-10-05 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-05.xlsx
+++ b/gex_pivot_levels_2026-10-05.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -610,12 +610,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$8.13M</t>
+          <t>-$8.62M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$8.73M</t>
+          <t>+$9.23M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -742,12 +742,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-$4.50M</t>
+          <t>-$4.62M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$7.23M</t>
+          <t>+$7.42M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -771,12 +771,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$17.99M</t>
+          <t>-$18.34M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$19.64M</t>
+          <t>+$20.03M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>-$5.96M</t>
+          <t>-$6.06M</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>+$12.54M</t>
+          <t>+$12.74M</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -870,12 +870,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>-$11.90M</t>
+          <t>-$12.21M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$18.26M</t>
+          <t>+$18.74M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>-$3.26M</t>
+          <t>-$3.30M</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>+$9.76M</t>
+          <t>+$9.88M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -969,12 +969,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>-$11.67M</t>
+          <t>-$11.81M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$43.28M</t>
+          <t>+$43.80M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>+$2.01M</t>
+          <t>+$1.98M</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+$8.62M</t>
+          <t>+$8.51M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>+$10.23M</t>
+          <t>+$10.06M</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>+$25.64M</t>
+          <t>+$25.23M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$2.50M</t>
+          <t>+$2.45M</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>+$5.64M</t>
+          <t>+$5.53M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1233,12 +1233,12 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>+$9.81M</t>
+          <t>+$9.32M</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>+$11.75M</t>
+          <t>+$11.16M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1287,10 +1287,10 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>7842.78</v>
+        <v>7847.78</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>7795</v>
+        <v>7800</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
@@ -1299,60 +1299,23 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>+$1.89M</t>
+          <t>+$6.00M</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>+$1.91M</t>
+          <t>+$6.31M</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>7847.78</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>7800</v>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>+$6.86M</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>+$7.21M</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:G25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3557,7 +3520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3669,12 +3632,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>-$11.67M</t>
+          <t>-$11.81M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>+$43.28M</t>
+          <t>+$43.80M</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3783,12 +3746,12 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>+$10.23M</t>
+          <t>+$10.06M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$25.64M</t>
+          <t>+$25.23M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3897,12 +3860,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>-$17.99M</t>
+          <t>-$18.34M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>+$19.64M</t>
+          <t>+$20.03M</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3973,12 +3936,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>-$11.90M</t>
+          <t>-$12.21M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$18.26M</t>
+          <t>+$18.74M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -4235,12 +4198,12 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>-$5.96M</t>
+          <t>-$6.06M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>+$12.54M</t>
+          <t>+$12.74M</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -4293,76 +4256,76 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2836.92</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>282</v>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>+$6.75M</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>+$11.58M</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B21" s="2" t="n">
         <v>7817.78</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C21" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>+$9.81M</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>+$11.75M</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>+$9.32M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>+$11.16M</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>2836.92</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>282</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>+$6.75M</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>+$11.58M</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -4383,12 +4346,12 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-$3.26M</t>
+          <t>-$3.30M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$9.76M</t>
+          <t>+$9.88M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -4475,76 +4438,76 @@
       <c r="H24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7667.78</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7620</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>-$8.62M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>+$9.23M</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B26" s="5" t="n">
         <v>31217.56</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C26" s="5" t="n">
         <v>753</v>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>+$8.72M</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>+$8.84M</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>7673.77</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>760</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>-$2.96M</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>+$8.74M</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4553,24 +4516,24 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>7667.78</v>
+        <v>7673.77</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>7620</v>
+        <v>760</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>-$8.13M</t>
+          <t>-$2.96M</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+$8.73M</t>
+          <t>+$8.74M</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -4603,12 +4566,12 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>+$2.01M</t>
+          <t>+$1.98M</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>+$8.62M</t>
+          <t>+$8.51M</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -4641,12 +4604,12 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>-$4.50M</t>
+          <t>-$4.62M</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>+$7.23M</t>
+          <t>+$7.42M</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -4657,80 +4620,76 @@
       <c r="H29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>7847.78</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>+$6.86M</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>+$7.21M</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2867.1</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>285</v>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>+$3.94M</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>+$6.54M</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>2867.1</v>
+        <v>7847.78</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>285</v>
+        <v>7800</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>+$3.94M</t>
+          <t>+$6.00M</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>+$6.54M</t>
+          <t>+$6.31M</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -4751,12 +4710,12 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>+$2.50M</t>
+          <t>+$2.45M</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>+$5.64M</t>
+          <t>+$5.53M</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -5077,28 +5036,28 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>7842.78</v>
+        <v>31258.66</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>7795</v>
+        <v>754</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>+$1.89M</t>
+          <t>+$1.51M</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>+$1.91M</t>
+          <t>+$1.77M</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -5115,146 +5074,146 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4148.51</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>378</v>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>-$311.88K</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>+$1.41M</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>88.47</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>-$1.11M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$1.39M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n">
-        <v>31258.66</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>754</v>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="B44" s="5" t="n">
+        <v>31464.16</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>759</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>+$1.51M</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>+$1.77M</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>+$1.17M</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>+$1.18M</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B43" s="5" t="n">
-        <v>4148.51</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>378</v>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="B45" s="2" t="n">
+        <v>4192.41</v>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>382</v>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>-$311.88K</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>+$1.41M</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>88.47</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>145</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>-$1.11M</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$1.39M</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>31464.16</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>759</v>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>+$1.17M</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>+$1.18M</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>-$75.17K</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>+$1.15M</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -5267,24 +5226,24 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>4192.41</v>
+        <v>4325.04</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>382</v>
+        <v>91</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>-$75.17K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>+$748.87K</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$1.15M</t>
+          <t>+$972.27K</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -5294,191 +5253,191 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n">
-        <v>4325.04</v>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="B47" s="5" t="n">
+        <v>4182.46</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
-          <t>+$748.87K</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>+$972.27K</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>+$7.46K</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>+$950.23K</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>7633.63</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>756</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>-$407.79K</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>+$931.76K</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n">
-        <v>4182.46</v>
-      </c>
-      <c r="C48" s="5" t="n">
-        <v>88</v>
-      </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="B49" s="2" t="n">
+        <v>3802.23</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>+$7.46K</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>+$950.23K</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="n">
-        <v>7633.63</v>
-      </c>
-      <c r="C49" s="5" t="n">
-        <v>756</v>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>-$407.79K</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>+$931.76K</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>-$894.13K</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>+$922.01K</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>31269.07</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>+$754.18K</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>+$828.12K</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n">
-        <v>3802.23</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>-$894.13K</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>+$922.01K</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>31269.07</v>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>31000</v>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>+$754.18K</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>+$828.12K</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="B51" s="5" t="n">
+        <v>4181.44</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>381</v>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>+$234.70K</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>+$804.76K</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5491,240 +5450,240 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>4181.44</v>
+        <v>4467.62</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>381</v>
+        <v>94</v>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>-$165.36K</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>+$742.16K</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>91.52</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>+$495.97K</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$676.48K</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4225.34</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>385</v>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>+$234.70K</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>+$804.76K</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>4467.62</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>94</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>-$165.36K</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$742.16K</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>+$194.04K</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>+$602.12K</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="H54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
-        <v>91.52</v>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="B55" s="2" t="n">
+        <v>82.37</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>+$495.97K</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>+$676.48K</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="n">
-        <v>4225.34</v>
-      </c>
-      <c r="C55" s="5" t="n">
-        <v>385</v>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>+$194.04K</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>+$602.12K</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>-$571.47K</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>+$576.63K</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>31069.07</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>30800</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>+$280.35K</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>+$568.71K</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n">
-        <v>82.37</v>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>135</v>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="B57" s="2" t="n">
+        <v>85.42</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>-$571.47K</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>+$576.63K</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>-$545.13K</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>+$558.75K</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="n">
-        <v>31069.07</v>
-      </c>
-      <c r="C57" s="5" t="n">
-        <v>30800</v>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>+$280.35K</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>+$568.71K</t>
-        </is>
-      </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>85.42</v>
+        <v>31169.07</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>140</v>
+        <v>30900</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>-$545.13K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>+$424.53K</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>+$558.75K</t>
+          <t>+$552.69K</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -5734,35 +5693,35 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>31169.07</v>
+        <v>4280.21</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>30900</v>
+        <v>390</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>+$424.53K</t>
+          <t>+$326.72K</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$552.69K</t>
+          <t>+$511.33K</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -5779,150 +5738,150 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>+$83.14K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$511.23K</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>89.08</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>146</v>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>+$257.73K</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>+$492.44K</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>31119.07</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>30850</v>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>+$276.04K</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>+$465.82K</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B60" s="2" t="n">
-        <v>4280.21</v>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>390</v>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="B63" s="5" t="n">
+        <v>4159.49</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>+$326.72K</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>+$511.33K</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>143</v>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>+$83.14K</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>+$511.23K</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="n">
-        <v>89.08</v>
-      </c>
-      <c r="C62" s="5" t="n">
-        <v>146</v>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>+$257.73K</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>+$492.44K</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>-$213.35K</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>+$451.74K</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="n">
-        <v>31119.07</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>30850</v>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>+$276.04K</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>+$465.82K</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5935,62 +5894,58 @@
         </is>
       </c>
       <c r="B64" s="5" t="n">
-        <v>4159.49</v>
+        <v>4372.57</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>379</v>
+        <v>92</v>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>-$213.35K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>+$252.34K</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>+$451.74K</t>
+          <t>+$443.45K</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B65" s="5" t="n">
-        <v>4372.57</v>
+        <v>94.58</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>92</v>
+        <v>155</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>+$252.34K</t>
+          <t>+$193.79K</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>+$443.45K</t>
+          <t>+$403.37K</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -6003,184 +5958,188 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B66" s="5" t="n">
-        <v>94.58</v>
+        <v>31059.07</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>155</v>
+        <v>30790</v>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>+$193.79K</t>
+          <t>+$284.36K</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>+$403.37K</t>
+          <t>+$364.46K</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>92.75</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>152</v>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>-$5.61K</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>+$293.47K</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>97.63</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>+$279.00K</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>+$286.97K</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>4335.09</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>395</v>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>+$248.49K</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>+$265.27K</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B67" s="5" t="n">
-        <v>31059.07</v>
-      </c>
-      <c r="C67" s="5" t="n">
-        <v>30790</v>
-      </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="B70" s="2" t="n">
+        <v>30969.07</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>30700</v>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>+$284.36K</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>+$364.46K</t>
-        </is>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="n">
-        <v>92.75</v>
-      </c>
-      <c r="C68" s="5" t="n">
-        <v>152</v>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E68" s="7" t="inlineStr">
-        <is>
-          <t>-$5.61K</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>+$293.47K</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H68" s="6" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>-$125.70K</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>+$221.82K</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n">
-        <v>97.63</v>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>160</v>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>+$279.00K</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>+$286.97K</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="n">
-        <v>4335.09</v>
-      </c>
-      <c r="C70" s="5" t="n">
-        <v>395</v>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>+$248.49K</t>
-        </is>
-      </c>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>+$265.27K</t>
-        </is>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H70" s="6" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -6189,24 +6148,24 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>30969.07</v>
+        <v>31019.07</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>30700</v>
+        <v>30750</v>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>-$125.70K</t>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>+$100.13K</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>+$221.82K</t>
+          <t>+$220.28K</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -6216,85 +6175,81 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>89.69</v>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>-$154.25K</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>+$204.54K</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n">
-        <v>31019.07</v>
-      </c>
-      <c r="C72" s="2" t="n">
-        <v>30750</v>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E72" s="9" t="inlineStr">
-        <is>
-          <t>+$100.13K</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>+$220.28K</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B73" s="5" t="n">
-        <v>89.69</v>
+        <v>31144.07</v>
       </c>
       <c r="C73" s="5" t="n">
-        <v>147</v>
+        <v>30875</v>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E73" s="7" t="inlineStr">
-        <is>
-          <t>-$154.25K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>+$148.19K</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>+$204.54K</t>
+          <t>+$164.21K</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -6303,10 +6258,10 @@
         </is>
       </c>
       <c r="B74" s="5" t="n">
-        <v>31144.07</v>
+        <v>31089.07</v>
       </c>
       <c r="C74" s="5" t="n">
-        <v>30875</v>
+        <v>30820</v>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
@@ -6315,12 +6270,12 @@
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>+$148.19K</t>
+          <t>+$80.10K</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>+$164.21K</t>
+          <t>+$136.17K</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -6337,10 +6292,10 @@
         </is>
       </c>
       <c r="B75" s="5" t="n">
-        <v>31089.07</v>
+        <v>30949.07</v>
       </c>
       <c r="C75" s="5" t="n">
-        <v>30820</v>
+        <v>30680</v>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
@@ -6349,12 +6304,12 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>+$80.10K</t>
+          <t>+$18.48K</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>+$136.17K</t>
+          <t>+$122.00K</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -6371,24 +6326,24 @@
         </is>
       </c>
       <c r="B76" s="5" t="n">
-        <v>30949.07</v>
+        <v>30899.07</v>
       </c>
       <c r="C76" s="5" t="n">
-        <v>30680</v>
+        <v>30630</v>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>+$18.48K</t>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-$88.11K</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>+$122.00K</t>
+          <t>+$115.22K</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
@@ -6401,74 +6356,74 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B77" s="5" t="n">
-        <v>30899.07</v>
+        <v>3944.82</v>
       </c>
       <c r="C77" s="5" t="n">
-        <v>30630</v>
+        <v>83</v>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>-$88.11K</t>
+          <t>-$100.50K</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>+$115.22K</t>
+          <t>+$104.61K</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H77" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B78" s="5" t="n">
-        <v>3944.82</v>
+        <v>31219.07</v>
       </c>
       <c r="C78" s="5" t="n">
-        <v>83</v>
+        <v>30950</v>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="inlineStr">
-        <is>
-          <t>-$100.50K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>+$29.58K</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>+$104.61K</t>
+          <t>+$81.33K</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
@@ -6477,32 +6432,36 @@
         </is>
       </c>
       <c r="B79" s="5" t="n">
-        <v>31219.07</v>
+        <v>31049.07</v>
       </c>
       <c r="C79" s="5" t="n">
-        <v>30950</v>
+        <v>30780</v>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>+$29.58K</t>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>-$40.05K</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>+$81.33K</t>
+          <t>+$80.10K</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H79" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
@@ -6511,10 +6470,10 @@
         </is>
       </c>
       <c r="B80" s="5" t="n">
-        <v>31049.07</v>
+        <v>31094.07</v>
       </c>
       <c r="C80" s="5" t="n">
-        <v>30780</v>
+        <v>30825</v>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
@@ -6523,12 +6482,12 @@
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>-$40.05K</t>
+          <t>-$56.07K</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>+$80.10K</t>
+          <t>+$72.09K</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr">
@@ -6545,28 +6504,28 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B81" s="5" t="n">
-        <v>31094.07</v>
+        <v>4301.28</v>
       </c>
       <c r="C81" s="5" t="n">
-        <v>30825</v>
+        <v>90.5</v>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="inlineStr">
-        <is>
-          <t>-$56.07K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>+$3.60K</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>+$72.09K</t>
+          <t>+$67.21K</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
@@ -6583,28 +6542,28 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B82" s="5" t="n">
-        <v>4301.28</v>
+        <v>30944.07</v>
       </c>
       <c r="C82" s="5" t="n">
-        <v>90.5</v>
+        <v>30675</v>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>+$3.60K</t>
+          <t>+$59.15K</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>+$67.21K</t>
+          <t>+$66.55K</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
@@ -6614,7 +6573,7 @@
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -6625,10 +6584,10 @@
         </is>
       </c>
       <c r="B83" s="5" t="n">
-        <v>30944.07</v>
+        <v>31129.07</v>
       </c>
       <c r="C83" s="5" t="n">
-        <v>30675</v>
+        <v>30860</v>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
@@ -6637,12 +6596,12 @@
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>+$59.15K</t>
+          <t>+$25.88K</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>+$66.55K</t>
+          <t>+$60.38K</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
@@ -6652,7 +6611,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -6663,24 +6622,24 @@
         </is>
       </c>
       <c r="B84" s="5" t="n">
-        <v>31129.07</v>
+        <v>31194.07</v>
       </c>
       <c r="C84" s="5" t="n">
-        <v>30860</v>
+        <v>30925</v>
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E84" s="8" t="inlineStr">
-        <is>
-          <t>+$25.88K</t>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-$4.01K</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>+$60.38K</t>
+          <t>+$28.04K</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
@@ -6697,28 +6656,28 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B85" s="5" t="n">
-        <v>31194.07</v>
+        <v>84.2</v>
       </c>
       <c r="C85" s="5" t="n">
-        <v>30925</v>
+        <v>138</v>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>-$4.01K</t>
+          <t>-$21.47K</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>+$28.04K</t>
+          <t>+$23.55K</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -6728,35 +6687,35 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B86" s="5" t="n">
-        <v>84.2</v>
+        <v>3849.76</v>
       </c>
       <c r="C86" s="5" t="n">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>-$21.47K</t>
+          <t>-$6.71K</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>+$23.55K</t>
+          <t>+$8.15K</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr">
@@ -6770,46 +6729,8 @@
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="n">
-        <v>3849.76</v>
-      </c>
-      <c r="C87" s="5" t="n">
-        <v>81</v>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E87" s="7" t="inlineStr">
-        <is>
-          <t>-$6.71K</t>
-        </is>
-      </c>
-      <c r="F87" s="6" t="inlineStr">
-        <is>
-          <t>+$8.15K</t>
-        </is>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H87"/>
+  <autoFilter ref="A1:H86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports 2026-10-05 10:42
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-05.xlsx
+++ b/gex_pivot_levels_2026-10-05.xlsx
@@ -610,12 +610,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$8.62M</t>
+          <t>-$6.23M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$9.23M</t>
+          <t>+$6.66M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -676,12 +676,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$1.37M</t>
+          <t>-$945.26K</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$2.72M</t>
+          <t>+$1.88M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -729,62 +729,66 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7697.78</v>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="n">
+        <v>7712.78</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7665</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>-$4.62M</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>+$7.42M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-$13.76M</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>+$15.02M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>7712.78</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>7665</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-$18.34M</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>+$20.03M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="A9" s="5" t="n">
+        <v>7713.91</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>764</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>-$3.13M</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>+$11.75M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -792,24 +796,24 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>7713.91</v>
+        <v>7722.78</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>764</v>
+        <v>7675</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$3.13M</t>
+          <t>-$4.88M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$11.75M</t>
+          <t>+$10.28M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -819,228 +823,228 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>7737.78</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>7690</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-$10.47M</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>+$16.07M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>7722.78</v>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>7675</v>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>7742.78</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>7695</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>-$6.06M</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>+$12.74M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>-$2.94M</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>+$8.79M</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>7737.78</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>7690</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>-$12.21M</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>+$18.74M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>7742.78</v>
+        <v>7744.01</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7695</v>
+        <v>767</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>+$4.00M</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>+$15.59M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7747.78</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>7700</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>-$3.30M</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>+$9.88M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-$10.82M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$40.15M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7764.08</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>769</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>+$1.04M</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>+$21.75M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>7744.01</v>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>767</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>7774.11</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>770</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>+$4.00M</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>+$15.59M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>7747.78</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>7700</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>-$11.81M</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+$43.80M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>7764.08</v>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>769</v>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>+$1.04M</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>+$21.75M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>+$12.18M</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>+$31.97M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>7774.11</v>
+        <v>7777.78</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>770</v>
+        <v>7730</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>+$12.18M</t>
+          <t>+$12.66M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$31.97M</t>
+          <t>+$27.95M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1055,264 +1059,268 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>7777.78</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7730</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="A18" s="5" t="n">
+        <v>7787.78</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7740</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>+$11.04M</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>+$24.38M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>+$2.44M</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>+$10.49M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>7787.78</v>
+        <v>7794.18</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>7740</v>
+        <v>772</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>+$6.26M</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>+$9.61M</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>7797.78</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>+$1.98M</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>+$8.51M</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>+$12.99M</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>+$32.56M</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>7807.78</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>7760</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>+$3.24M</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>+$7.29M</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>7794.18</v>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>772</v>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>+$6.26M</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>+$9.61M</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>7797.78</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>7817.78</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>7770</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>+$10.06M</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>+$25.23M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>7807.78</v>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>7760</v>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>+$2.45M</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>+$5.53M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>+$12.51M</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>+$14.98M</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>7817.78</v>
+        <v>7824.28</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>7770</v>
+        <v>775</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>+$12.07M</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>+$15.71M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>7842.78</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7795</v>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>+$9.32M</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>+$11.16M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>7824.28</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>775</v>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>+$12.07M</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>+$15.71M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>+$2.08M</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>+$2.11M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="2" t="n">
         <v>7847.78</v>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B25" s="2" t="n">
         <v>7800</v>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>+$6.00M</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>+$6.31M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr"/>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>+$7.73M</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>+$8.10M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G25"/>
@@ -3632,12 +3640,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>-$11.81M</t>
+          <t>-$10.82M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>+$43.80M</t>
+          <t>+$40.15M</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3658,24 +3666,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>7774.11</v>
+        <v>7797.78</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>770</v>
+        <v>7750</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>+$12.18M</t>
+          <t>+$12.99M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$31.97M</t>
+          <t>+$32.56M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3692,28 +3700,28 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>30518.86</v>
+        <v>7774.11</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>736</v>
+        <v>770</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>-$26.10M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>+$12.18M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$27.31M</t>
+          <t>+$31.97M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3723,7 +3731,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3734,10 +3742,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7797.78</v>
+        <v>7777.78</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>7750</v>
+        <v>7730</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -3746,12 +3754,12 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>+$10.06M</t>
+          <t>+$12.66M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$25.23M</t>
+          <t>+$27.95M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3768,28 +3776,28 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>7777.78</v>
+        <v>30518.86</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7730</v>
+        <v>736</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>+$11.04M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>-$26.10M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>+$24.38M</t>
+          <t>+$27.31M</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -3799,7 +3807,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3844,28 +3852,28 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>7712.78</v>
+        <v>2857.04</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7665</v>
+        <v>284</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>-$18.34M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>+$18.18M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>+$20.03M</t>
+          <t>+$19.08M</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3875,35 +3883,35 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>2857.04</v>
+        <v>31505.26</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>284</v>
+        <v>760</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>+$18.18M</t>
+          <t>+$18.08M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>+$19.08M</t>
+          <t>+$18.09M</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3920,28 +3928,28 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>7737.78</v>
+        <v>31094.26</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7690</v>
+        <v>750</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>-$12.21M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>+$16.15M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$18.74M</t>
+          <t>+$17.70M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -3951,35 +3959,35 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>31505.26</v>
+        <v>7737.78</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>760</v>
+        <v>7690</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>+$18.08M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>-$10.47M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+$18.09M</t>
+          <t>+$16.07M</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3989,35 +3997,35 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>31094.26</v>
+        <v>7824.28</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>750</v>
+        <v>775</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>+$16.15M</t>
+          <t>+$12.07M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$17.70M</t>
+          <t>+$15.71M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -4032,38 +4040,38 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
-        <v>7824.28</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>775</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="B14" s="5" t="n">
+        <v>7744.01</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>767</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$12.07M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$15.71M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>+$4.00M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>+$15.59M</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4072,146 +4080,146 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2816.8</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>280</v>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>+$8.03M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>+$15.40M</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
-        <v>7744.01</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>767</v>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>+$4.00M</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>+$15.59M</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>2816.8</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>280</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>+$8.03M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$15.40M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="B16" s="2" t="n">
+        <v>7712.78</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>7665</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>-$13.76M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>+$15.02M</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>7817.78</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>7770</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>+$12.51M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>+$14.98M</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B18" s="2" t="n">
         <v>2877.16</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C18" s="2" t="n">
         <v>286</v>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>+$14.21M</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>+$14.60M</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>7722.78</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>7675</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>-$6.06M</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>+$12.74M</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4290,40 +4298,40 @@
       <c r="H20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
-        <v>7817.78</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>7770</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="B21" s="5" t="n">
+        <v>7787.78</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>7740</v>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>+$9.32M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>+$11.16M</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>+$2.44M</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>+$10.49M</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4334,10 +4342,10 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7742.78</v>
+        <v>7722.78</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>7695</v>
+        <v>7675</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -4346,12 +4354,12 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-$3.30M</t>
+          <t>-$4.88M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$9.88M</t>
+          <t>+$10.28M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -4438,76 +4446,76 @@
       <c r="H24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>7667.78</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>7620</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-$8.62M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$9.23M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>31217.56</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>753</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$8.72M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$8.84M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>31217.56</v>
+        <v>7742.78</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>753</v>
+        <v>7695</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$8.72M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>-$2.94M</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>+$8.84M</t>
+          <t>+$8.79M</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4548,40 +4556,40 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>7787.78</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>7740</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="B28" s="2" t="n">
+        <v>7847.78</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>+$1.98M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$8.51M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>+$7.73M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$8.10M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4592,66 +4600,70 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>7697.78</v>
+        <v>7807.78</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>7650</v>
+        <v>7760</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>-$4.62M</t>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>+$3.24M</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>+$7.42M</t>
+          <t>+$7.29M</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>2867.1</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>285</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>+$3.94M</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>+$6.54M</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>7667.78</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>7620</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>-$6.23M</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>+$6.66M</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4660,36 +4672,40 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7847.78</v>
+        <v>2867.1</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>7800</v>
+        <v>285</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>+$6.00M</t>
+          <t>+$3.94M</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>+$6.31M</t>
+          <t>+$6.54M</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -4698,24 +4714,24 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>7807.78</v>
+        <v>7683.8</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>7760</v>
+        <v>761</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>+$2.45M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>-$91.91K</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>+$5.53M</t>
+          <t>+$4.96M</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -4725,43 +4741,43 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>7683.8</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>761</v>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>-$91.91K</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>+$4.96M</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>4277.51</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>+$1.07M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$3.82M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4774,24 +4790,24 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>4277.51</v>
+        <v>4039.87</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>+$1.07M</t>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>-$3.35M</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>+$3.82M</t>
+          <t>+$3.64M</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -4801,35 +4817,35 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>4039.87</v>
+        <v>7623.6</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>85</v>
+        <v>755</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>-$3.35M</t>
+          <t>-$2.91M</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>+$3.64M</t>
+          <t>+$3.37M</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -4846,112 +4862,112 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>4170.46</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>-$833.99K</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>+$2.58M</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>4115.59</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>-$1.71M</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>+$2.27M</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
-        <v>7623.6</v>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>755</v>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>-$2.91M</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>+$3.37M</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>7682.78</v>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>7635</v>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="B38" s="5" t="n">
+        <v>7842.78</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>7795</v>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>-$1.37M</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>+$2.72M</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>+$2.08M</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>+$2.11M</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>4170.46</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>380</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>-$833.99K</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>+$2.58M</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4964,24 +4980,24 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>4115.59</v>
+        <v>3897.29</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>375</v>
+        <v>82</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>-$1.71M</t>
+          <t>-$2.00M</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>+$2.27M</t>
+          <t>+$2.00M</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -4996,40 +5012,40 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>3897.29</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>-$2.00M</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>+$2.00M</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>7682.78</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>7635</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>-$945.26K</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>+$1.88M</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>

</xml_diff>